<commit_message>
Updated Uploads Page & added more subjects & added confetti for pass
</commit_message>
<xml_diff>
--- a/RESULTS/2017/CLASS/SS1/Chemistry/results.xlsx
+++ b/RESULTS/2017/CLASS/SS1/Chemistry/results.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,108 +413,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Student Name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Admission No</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Subject</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Score (%)</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Time Taken</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Submitted At</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Imogdabe Mariam Medinah</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>std189</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>SS1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>CHEMISTRY</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>4%</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>4</v>
-      </c>
-      <c r="G2" t="n">
-        <v>50</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>2025-12-12 08:22</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>